<commit_message>
fix(xiao): C17 to Murata GRM21BR61E226ME44L (LCSC C86816)
User-selected at JLC assembly order; prior C398931 unavailable in their
matcher. Same 22uF/25V/X5R/0805 class, verified on JLC part page.
Regenerated xlsx and JLC-format BOMs from the CSV source.
</commit_message>
<xml_diff>
--- a/Custom PCB esp32c6/fab-xiao/BOM_xiao.xlsx
+++ b/Custom PCB esp32c6/fab-xiao/BOM_xiao.xlsx
@@ -540,7 +540,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>GRT21BR61E226ME13L</t>
+          <t>GRM21BR61E226ME44L</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -555,12 +555,12 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>DigiKey 490-GRT21BR61E226ME13LCT-ND</t>
+          <t>DigiKey/Mouser: search MPN GRM21BR61E226ME44L</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Buck V_in cap; replaces obsolete/OOS C45783</t>
+          <t>Buck V_in cap; user-selected C86816 at JLC order 2026-07-21 (prior C398931 unavailable in matcher); same 22uF/25V/X5R/0805 class</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(xiao): sync BOM to as-ordered JLC assembly parts
Order finalized 2026-07-21, 5 boards. Fee-free swaps verified by research
pass: D2/D3 H5VL10B (5V bidir 15pF), D5 Hongjiacheng SMF15A, D6 B0520W
(Vf~385mV parametric, datasheet check flagged). C17/C19/R8/R10/R11 moved
to in-stock Basic parts, R8 corrected to 30k after a 1k mismatch in the
matcher. C15 stays Murata C2292827 (only 47uF/10V option with published
DC-bias data). Original design parts retained in notes as DigiKey
sourceable alternates. Placement-preview polarity check passed for
D5/D6/U1/Q1 against board pad nets.
</commit_message>
<xml_diff>
--- a/Custom PCB esp32c6/fab-xiao/BOM_xiao.xlsx
+++ b/Custom PCB esp32c6/fab-xiao/BOM_xiao.xlsx
@@ -535,12 +535,12 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Murata</t>
+          <t>Samsung Electro-Mechanics</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>GRM21BR61E226ME44L</t>
+          <t>CL21A226MAQNNNE</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -560,7 +560,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Buck V_in cap; user-selected C86816 at JLC order 2026-07-21 (prior C398931 unavailable in matcher); same 22uF/25V/X5R/0805 class</t>
+          <t>Buck V_in cap; user-selected C86816 at JLC order 2026-07-21 (prior C398931 unavailable in matcher); same 22uF/25V/X5R/0805 class; as-ordered JLC 2026-07-21: JLC Basic; prior picks GRT21BR61E226ME13L/GRM21BR61E226ME44L remain valid alternates</t>
         </is>
       </c>
     </row>
@@ -664,12 +664,12 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Samsung Electro-Mechanics</t>
+          <t>Fenghua</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>CL05C470JB5NNNC</t>
+          <t>0402CG470J500NT</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -689,7 +689,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Buck feedforward across R6; replaces wrong C1549 (18pF)</t>
+          <t>Buck feedforward across R6; replaces wrong C1549 (18pF); as-ordered JLC 2026-07-21: JLC Basic; design part Samsung CL05C470JB5NNNC (C84706) = DK-sourceable alternate</t>
         </is>
       </c>
     </row>
@@ -750,12 +750,12 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>GOODWORK</t>
+          <t>Hongjiacheng</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>ES05D1MC10</t>
+          <t>H5VL10B</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -775,7 +775,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>S21 TX line-to-GND protection; 5V standoff, 11V clamp, 8A/80W. GOODWORK is an LCSC-house brand; no direct DigiKey/Mouser cross</t>
+          <t>S21 TX line-to-GND protection; 5V standoff, 11V clamp, 8A/80W. GOODWORK is an LCSC-house brand; no direct DigiKey/Mouser cross; as-ordered JLC 2026-07-21: fee-free swap, 5V bidir 15pF DFN1006-2L; design part ES05D1MC10 (C5137770) = alternate</t>
         </is>
       </c>
     </row>
@@ -793,7 +793,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>MDD (Microdiode)</t>
+          <t>Hongjiacheng</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -818,7 +818,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Input TVS, 15V standoff. LCSC primary C123802 is MDD-brand SMF15A; the DK number is a Littelfuse cross-substitution (verified: F5817CT-ND = Littelfuse SMF15A, SOD-123F, 15V standoff / 24.4V clamp)</t>
+          <t>Input TVS, 15V standoff. LCSC primary C123802 is MDD-brand SMF15A; the DK number is a Littelfuse cross-substitution (verified: F5817CT-ND = Littelfuse SMF15A, SOD-123F, 15V standoff / 24.4V clamp); as-ordered JLC 2026-07-21: fee-free brand swap, same SMF15A spec; MDD C123802 / Littelfuse F5817CT-ND = alternates</t>
         </is>
       </c>
     </row>
@@ -836,12 +836,12 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Nexperia</t>
+          <t>Hongjiacheng</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>PMEG2005EH,115</t>
+          <t>B0520W</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -861,7 +861,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>USB VBUS isolation; SOD-123F land-compatible with the D_SOD-123 footprint. DK 1157665 backorder as of 2026-07-20; LCSC C96233 in stock</t>
+          <t>USB VBUS isolation; SOD-123F land-compatible with the D_SOD-123 footprint. DK 1157665 backorder as of 2026-07-20; LCSC C96233 in stock; as-ordered JLC 2026-07-21: fee-free swap, 20V Schottky Vf~385mV@0.5A (JLC parametric); design part PMEG2005EH (C96233) = alternate</t>
         </is>
       </c>
     </row>
@@ -1176,12 +1176,12 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>YAGEO</t>
+          <t>UNI-ROYAL</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>RC0402FR-0730KL</t>
+          <t>0402WGF3002TCE</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1201,7 +1201,7 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Buck feedback bottom; sets Vout=5.0V. Replaces wrong C25779 (33k) and OOS C25776</t>
+          <t>Buck feedback bottom; sets Vout=5.0V. Replaces wrong C25779 (33k) and OOS C25776; as-ordered JLC 2026-07-21: restocked; design part YAGEO RC0402FR-0730KL (C138008) = DK-sourceable alternate</t>
         </is>
       </c>
     </row>
@@ -1224,7 +1224,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>0603WAJ0221T5E</t>
+          <t>0603WAF2200T5E</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1244,7 +1244,7 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>S21 series resistor</t>
+          <t>S21 series resistor; as-ordered JLC 2026-07-21: 1% part supersedes 5% C1226; JLC Basic</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(xiao): correct order status to cart-staged, not placed
The JLC walkthrough was a part-picking exercise; no order has been
placed. Prior commit dc99918's 'order finalized' wording overclaimed.
Part selections remain valid; stock and matcher results must be
re-verified at actual order time.
</commit_message>
<xml_diff>
--- a/Custom PCB esp32c6/fab-xiao/BOM_xiao.xlsx
+++ b/Custom PCB esp32c6/fab-xiao/BOM_xiao.xlsx
@@ -560,7 +560,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Buck V_in cap; user-selected C86816 at JLC order 2026-07-21 (prior C398931 unavailable in matcher); same 22uF/25V/X5R/0805 class; as-ordered JLC 2026-07-21: JLC Basic; prior picks GRT21BR61E226ME13L/GRM21BR61E226ME44L remain valid alternates</t>
+          <t>Buck V_in cap; user-selected C86816 at JLC order 2026-07-21 (prior C398931 unavailable in matcher); same 22uF/25V/X5R/0805 class; JLC cart selection 2026-07-21 (order not yet placed): JLC Basic; prior picks GRT21BR61E226ME13L/GRM21BR61E226ME44L remain valid alternates</t>
         </is>
       </c>
     </row>
@@ -689,7 +689,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Buck feedforward across R6; replaces wrong C1549 (18pF); as-ordered JLC 2026-07-21: JLC Basic; design part Samsung CL05C470JB5NNNC (C84706) = DK-sourceable alternate</t>
+          <t>Buck feedforward across R6; replaces wrong C1549 (18pF); JLC cart selection 2026-07-21 (order not yet placed): JLC Basic; design part Samsung CL05C470JB5NNNC (C84706) = DK-sourceable alternate</t>
         </is>
       </c>
     </row>
@@ -775,7 +775,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>S21 TX line-to-GND protection; 5V standoff, 11V clamp, 8A/80W. GOODWORK is an LCSC-house brand; no direct DigiKey/Mouser cross; as-ordered JLC 2026-07-21: fee-free swap, 5V bidir 15pF DFN1006-2L; design part ES05D1MC10 (C5137770) = alternate</t>
+          <t>S21 TX line-to-GND protection; 5V standoff, 11V clamp, 8A/80W. GOODWORK is an LCSC-house brand; no direct DigiKey/Mouser cross; JLC cart selection 2026-07-21 (order not yet placed): fee-free swap, 5V bidir 15pF DFN1006-2L; design part ES05D1MC10 (C5137770) = alternate</t>
         </is>
       </c>
     </row>
@@ -818,7 +818,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Input TVS, 15V standoff. LCSC primary C123802 is MDD-brand SMF15A; the DK number is a Littelfuse cross-substitution (verified: F5817CT-ND = Littelfuse SMF15A, SOD-123F, 15V standoff / 24.4V clamp); as-ordered JLC 2026-07-21: fee-free brand swap, same SMF15A spec; MDD C123802 / Littelfuse F5817CT-ND = alternates</t>
+          <t>Input TVS, 15V standoff. LCSC primary C123802 is MDD-brand SMF15A; the DK number is a Littelfuse cross-substitution (verified: F5817CT-ND = Littelfuse SMF15A, SOD-123F, 15V standoff / 24.4V clamp); JLC cart selection 2026-07-21 (order not yet placed): fee-free brand swap, same SMF15A spec; MDD C123802 / Littelfuse F5817CT-ND = alternates</t>
         </is>
       </c>
     </row>
@@ -861,7 +861,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>USB VBUS isolation; SOD-123F land-compatible with the D_SOD-123 footprint. DK 1157665 backorder as of 2026-07-20; LCSC C96233 in stock; as-ordered JLC 2026-07-21: fee-free swap, 20V Schottky; Vf verified from datasheet Fig.2: ~0.38V@0.5A, ~0.30V@0.15A typ 25C; design part PMEG2005EH (C96233) = alternate</t>
+          <t>USB VBUS isolation; SOD-123F land-compatible with the D_SOD-123 footprint. DK 1157665 backorder as of 2026-07-20; LCSC C96233 in stock; JLC cart selection 2026-07-21 (order not yet placed): fee-free swap, 20V Schottky; Vf verified from datasheet Fig.2: ~0.38V@0.5A, ~0.30V@0.15A typ 25C; design part PMEG2005EH (C96233) = alternate</t>
         </is>
       </c>
     </row>
@@ -1201,7 +1201,7 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Buck feedback bottom; sets Vout=5.0V. Replaces wrong C25779 (33k) and OOS C25776; as-ordered JLC 2026-07-21: restocked; design part YAGEO RC0402FR-0730KL (C138008) = DK-sourceable alternate</t>
+          <t>Buck feedback bottom; sets Vout=5.0V. Replaces wrong C25779 (33k) and OOS C25776; JLC cart selection 2026-07-21 (order not yet placed): restocked; design part YAGEO RC0402FR-0730KL (C138008) = DK-sourceable alternate</t>
         </is>
       </c>
     </row>
@@ -1244,7 +1244,7 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>S21 series resistor; as-ordered JLC 2026-07-21: 1% part supersedes 5% C1226; JLC Basic</t>
+          <t>S21 series resistor; JLC cart selection 2026-07-21 (order not yet placed): 1% part supersedes 5% C1226; JLC Basic</t>
         </is>
       </c>
     </row>

</xml_diff>